<commit_message>
chore(release): sync committed v4.5.2 artifacts with published assets
The committed workbook + manifest still carried v4.5.1 content. Update
them to the v4.5.2 build: the workbook regenerated at 4.5.2, and the
unified 11-asset SHA256SUMS that was uploaded to and remote-verified
against the v4.5.2 release. No version change, no code change.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -789,7 +789,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v4.5.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v4.5.2 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>4.5.0</t>
+          <t>4.5.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v4.7 A75/A79: public labelling + security/dual-use statements; sync artifacts
Adds the R33 public-metaphor labelling statement and the R35
security/privacy/dual-use analysis to the findings (this doc commit
lands one commit after the v4.7.0 tag; the GitHub release notes
already carry the public Boundary). Syncs the committed workbook and
unified 11-asset manifest to the published, remote-verified v4.7.0
build.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -27,7 +27,10 @@
     <sheet name="CSCP Tetrahedron" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="CSCP Spacetime" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="CSCP Experiments" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Workbook Guide" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="PMWR Recovery" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="PMWR Crystal" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="PMWR Phryll" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Workbook Guide" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,7 +67,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +126,51 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E8D8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0E0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A0E8A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E0C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0D0C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0D0D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0E0A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0E8E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D0F0D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="002E3A46"/>
       </patternFill>
     </fill>
@@ -139,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,10 +205,19 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -424,6 +481,23 @@
 </table>
 </file>
 
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="PMWRRecovery" displayName="PMWRRecovery" ref="A1:H5" headerRowCount="1">
+  <autoFilter ref="A1:H5"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="closure_window_s"/>
+    <tableColumn id="7" name="aliases_per_second"/>
+    <tableColumn id="8" name="statement"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HarmonicRelations" displayName="HarmonicRelations" ref="A1:M8" headerRowCount="1">
   <autoFilter ref="A1:M8"/>
@@ -441,6 +515,43 @@
     <tableColumn id="11" name="exact"/>
     <tableColumn id="12" name="abs_error_hz"/>
     <tableColumn id="13" name="note"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="PMWRCrystal" displayName="PMWRCrystal" ref="A1:J8" headerRowCount="1">
+  <autoFilter ref="A1:J8"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="theta_deg"/>
+    <tableColumn id="7" name="h_over_half_base"/>
+    <tableColumn id="8" name="full_base_over_height"/>
+    <tableColumn id="9" name="abs_diff_from_pi_over_2"/>
+    <tableColumn id="10" name="mechanism_claim"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="PMWRPhryll" displayName="PMWRPhryll" ref="A1:I15" headerRowCount="1">
+  <autoFilter ref="A1:I15"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="ladder"/>
+    <tableColumn id="7" name="detected_state_exists"/>
+    <tableColumn id="8" name="operator_note_sha256"/>
+    <tableColumn id="9" name="note_status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
 </table>
@@ -506,8 +617,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F105" headerRowCount="1">
-  <autoFilter ref="A1:F105"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F130" headerRowCount="1">
+  <autoFilter ref="A1:F130"/>
   <tableColumns count="6">
     <tableColumn id="1" name="table"/>
     <tableColumn id="2" name="id"/>
@@ -868,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -885,7 +996,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v4.6.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v4.7.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -1060,128 +1171,221 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>resonator_platform</t>
+          <t>pmwr_crystal</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>pmwr_phryll</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>specimens</t>
+          <t>pmwr_recovery</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>resonator_platform</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>specimens</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>timing_recipes</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B30" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B28" s="4">
-        <f>SUM(B10:B27)</f>
+      <c r="B31" s="4">
+        <f>SUM(B10:B30)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Evidence classes (weakest -&gt; strongest):</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>LORE</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>DERIVED_ARITHMETIC</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>ANALYTIC_MODEL</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>NUMERICAL_SIMULATION</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>SYNTHETIC_RUN</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>BENCH_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>INDEPENDENT_REPLICATION</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>NOT_APPLICABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>METAPHOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>CALIBRATED_MEASUREMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="inlineStr">
+        <is>
+          <t>ANTHROPOGENIC_STRUCTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>REPRESENTATION_ARTIFACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>CIRCULAR_DERIVATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>UNEXPLAINED_INSTRUMENT_RESIDUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>REPLICATED_ANOMALY</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>PROSPECTIVE_PREDICTION</t>
         </is>
       </c>
     </row>
@@ -1217,62 +1421,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>predicted_hz</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>target_hz</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>final_fitted_hz</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>accepted</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>iterations</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>synthetic</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>banner</t>
         </is>
@@ -1357,47 +1561,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>board</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>candidate_output_pins</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1707,42 +1911,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>campaign</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -2094,32 +2298,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>statement</t>
         </is>
@@ -2475,52 +2679,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>doi</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>publication_state</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>forbidden_transfers</t>
         </is>
@@ -2813,37 +3017,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>statement</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2918,62 +3122,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>product</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>install_scope</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>signed</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>telemetry</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>network</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>claim_boundary</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>version</t>
         </is>
@@ -3033,7 +3237,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>4.6.0</t>
+          <t>4.7.0</t>
         </is>
       </c>
     </row>
@@ -3069,62 +3273,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>exact_value</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>physically_supported_value</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>significant_figures</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>overclaims_if_quoted_exactly</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -4119,47 +4323,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>source_phrase</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>n_readings</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>resolution</t>
         </is>
@@ -4365,57 +4569,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>apparatus</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>energy_j</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>equivalent_mass_kg</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>schwarzschild_radius_m</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>orders_of_magnitude_below_proton</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>verdict</t>
         </is>
@@ -4664,47 +4868,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>hz</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>hz_float</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
@@ -5282,62 +5486,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>question</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>n_controls</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>n_per_condition</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>blinding</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>stopping_rule</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>apparatus_status</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>data_status</t>
         </is>
@@ -5473,6 +5677,1115 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>closure_window_s</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>aliases_per_second</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>PMWR-CLOSURE-ALIAS</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>ambiguity</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.recovery.closure_delay_ambiguity</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0.000244140625</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>4097</v>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>delays tau and tau + k*W are indistinguishable for every tone in this family; exact closure IS the alias (firewall CLOSURE_REMOVES_AMBIGUITY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>PMWR-DUAL-LATTICE</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>probe_design</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.recovery.dual_lattice_probe</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-TWO-GEODESIC</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>worldline_channel</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.worldline.two_geodesic_case</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="8" t="n"/>
+      <c r="H4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>PMWR-NOVELTY</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>novelty_boundary</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.ingest.NOVELTY_BOUNDARY</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>theta_deg</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>h_over_half_base</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>full_base_over_height</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>abs_diff_from_pi_over_2</t>
+        </is>
+      </c>
+      <c r="J1" s="24" t="inlineStr">
+        <is>
+          <t>mechanism_claim</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-360_over_7</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="n">
+        <v>51.42857142857143</v>
+      </c>
+      <c r="G2" s="16" t="n">
+        <v>1.253960337663</v>
+      </c>
+      <c r="H2" s="16" t="n">
+        <v>1.594946777765</v>
+      </c>
+      <c r="I2" s="16" t="n">
+        <v>0.024150451</v>
+      </c>
+      <c r="J2" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-51_843</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>51.843</v>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>1.272737633428</v>
+      </c>
+      <c r="H3" s="16" t="n">
+        <v>1.571415779239</v>
+      </c>
+      <c r="I3" s="16" t="n">
+        <v>0.000619452</v>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-51_51_51_DMS</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="n">
+        <v>51.86416666666667</v>
+      </c>
+      <c r="G4" s="16" t="n">
+        <v>1.273705938861</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>1.570221146797</v>
+      </c>
+      <c r="I4" s="16" t="n">
+        <v>0.00057518</v>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-Great_Pyramid_nominal</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>51.84</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>1.272600466963</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>1.57158515333</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>0.000788827</v>
+      </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-rounded_52</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>52</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>1.279941632193</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>1.562571253013</v>
+      </c>
+      <c r="I6" s="16" t="n">
+        <v>0.008225074000000001</v>
+      </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-emitter_58</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>58</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>1.600334529041</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>1.249738703819</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>0.321057623</v>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-emitter_60</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>1.732050807569</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>1.154700538379</v>
+      </c>
+      <c r="I8" s="16" t="n">
+        <v>0.416095788</v>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>REFUSED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>ladder</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>detected_state_exists</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>operator_note_sha256</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>note_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>PHRYLL-OPERATIONALIZATION</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>latent_definition</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>pack core/06; pmwr.crystal.PROMOTION_GATES</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM -&gt; OPERATIONAL_HYPOTHESIS -&gt; UNEXPLAINED_INSTRUMENT_RESIDUAL -&gt; REPLICATED_ANOMALY -&gt; CANDIDATE_NEW_MECHANISM</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>fff2f47e7c690eeda59fc6cc2d8e968d32a94f891155473aa65dbc592cb223d9</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>LORE,HYPOTHESIS_SEED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-PERFECT_ABSOLUTE_PHASE</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-ENVIRONMENTAL_IMMUNITY</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-ONE_RESIDUAL_ONE_PATH</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-CLOSURE_REMOVES_AMBIGUITY</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-4096_PRIVILEGED</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-PYRAMID_PROVES_MECHANISM</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-ANGLE_PROVES_DIRECTIONALITY</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-SENSOR_CHANGE_IS_PHRYLL</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-DEVICE_MIRACLES</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-REORDER_IS_REVERSAL</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-BENCH-DIRECTIONAL</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>bench_preregistration</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.benches</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-BENCH-SELFOSC</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>bench_preregistration</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.benches</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-BENCH-SHAM</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>bench_preregistration</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.benches</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5480,7 +6793,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Workbook Guide</t>
         </is>
@@ -5668,67 +6981,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>expression</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>output_hz</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>target_hz</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>primary_class</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="24" t="inlineStr">
         <is>
           <t>abs_error_hz</t>
         </is>
       </c>
-      <c r="M1" s="15" t="inlineStr">
+      <c r="M1" s="24" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -6206,57 +7519,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>revision</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>length_mm</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>facets</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>material_claim</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
@@ -6345,52 +7658,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>model_level</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>quarter_wave_hz</t>
         </is>
       </c>
-      <c r="E1" s="16" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>half_wave_hz</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="F1" s="25" t="inlineStr">
         <is>
           <t>target_hz</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="G1" s="25" t="inlineStr">
         <is>
           <t>rel_error_formula</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="H1" s="25" t="inlineStr">
         <is>
           <t>band_lo_hz</t>
         </is>
       </c>
-      <c r="I1" s="16" t="inlineStr">
+      <c r="I1" s="25" t="inlineStr">
         <is>
           <t>band_hi_hz</t>
         </is>
       </c>
-      <c r="J1" s="16" t="inlineStr">
+      <c r="J1" s="25" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -6465,57 +7778,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>family</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>frequency_hz</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>mechanism</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>order</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>hypothesis</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>is_control</t>
         </is>
@@ -7134,52 +8447,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>statement</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>mechanism</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>prediction</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>disconfirmed_by</t>
         </is>
@@ -7511,7 +8824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7523,32 +8836,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
@@ -10659,224 +11972,1024 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="inlineStr">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_recovery</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>PMWR-CLOSURE-ALIAS</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>ambiguity</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.recovery.closure_delay_ambiguity</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_recovery</t>
+        </is>
+      </c>
+      <c r="B100" s="7" t="inlineStr">
+        <is>
+          <t>PMWR-DUAL-LATTICE</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>probe_design</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.recovery.dual_lattice_probe</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>pmwr_recovery</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-TWO-GEODESIC</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>worldline_channel</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.worldline.two_geodesic_case</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_recovery</t>
+        </is>
+      </c>
+      <c r="B102" s="7" t="inlineStr">
+        <is>
+          <t>PMWR-NOVELTY</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>novelty_boundary</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E102" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F102" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.ingest.NOVELTY_BOUNDARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B103" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-360_over_7</t>
+        </is>
+      </c>
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E103" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F103" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B104" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-51_843</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B105" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-51_51_51_DMS</t>
+        </is>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D105" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F105" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B106" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-Great_Pyramid_nominal</t>
+        </is>
+      </c>
+      <c r="C106" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F106" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B107" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-rounded_52</t>
+        </is>
+      </c>
+      <c r="C107" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D107" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F107" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B108" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-emitter_58</t>
+        </is>
+      </c>
+      <c r="C108" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D108" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F108" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="16" t="inlineStr">
+        <is>
+          <t>pmwr_crystal</t>
+        </is>
+      </c>
+      <c r="B109" s="16" t="inlineStr">
+        <is>
+          <t>ANGLE-emitter_60</t>
+        </is>
+      </c>
+      <c r="C109" s="16" t="inlineStr">
+        <is>
+          <t>geometry_candidate</t>
+        </is>
+      </c>
+      <c r="D109" s="16" t="inlineStr">
+        <is>
+          <t>GEOMETRY_IDENTITY</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F109" s="16" t="inlineStr">
+        <is>
+          <t>pmwr.crystal.pyramid_ratio_audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>PHRYLL-OPERATIONALIZATION</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>latent_definition</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>pack core/06; pmwr.crystal.PROMOTION_GATES</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-PERFECT_ABSOLUTE_PHASE</t>
+        </is>
+      </c>
+      <c r="C111" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D111" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F111" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-ENVIRONMENTAL_IMMUNITY</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F112" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-ONE_RESIDUAL_ONE_PATH</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F113" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-CLOSURE_REMOVES_AMBIGUITY</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-4096_PRIVILEGED</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-PYRAMID_PROVES_MECHANISM</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-ANGLE_PROVES_DIRECTIONALITY</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-SENSOR_CHANGE_IS_PHRYLL</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-DEVICE_MIRACLES</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F119" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>FIREWALL-REORDER_IS_REVERSAL</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t>firewall</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F120" s="7" t="inlineStr">
+        <is>
+          <t>pmwr.FIREWALLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-BENCH-DIRECTIONAL</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>bench_preregistration</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F121" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.benches</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-BENCH-SELFOSC</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>bench_preregistration</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F122" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.benches</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
+          <t>pmwr_phryll</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>PMWR-BENCH-SHAM</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t>bench_preregistration</t>
+        </is>
+      </c>
+      <c r="D123" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E123" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F123" s="8" t="inlineStr">
+        <is>
+          <t>pmwr.benches</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B99" s="6" t="inlineStr">
+      <c r="B124" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-01</t>
         </is>
       </c>
-      <c r="C99" s="6" t="inlineStr">
+      <c r="C124" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D99" s="6" t="inlineStr">
+      <c r="D124" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E99" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="E124" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F124" s="6" t="inlineStr">
         <is>
           <t>local hash 019435a03b3c5e9d</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="6" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B125" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-02</t>
         </is>
       </c>
-      <c r="C100" s="6" t="inlineStr">
+      <c r="C125" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D100" s="6" t="inlineStr">
+      <c r="D125" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E100" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F100" s="6" t="inlineStr">
+      <c r="E125" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F125" s="6" t="inlineStr">
         <is>
           <t>local hash 7e1df086615c6bac</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="6" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B126" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-03</t>
         </is>
       </c>
-      <c r="C101" s="6" t="inlineStr">
+      <c r="C126" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr">
+      <c r="D126" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E101" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F101" s="6" t="inlineStr">
+      <c r="E126" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F126" s="6" t="inlineStr">
         <is>
           <t>local hash b8e387558cb0a0f0</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="6" t="inlineStr">
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B102" s="6" t="inlineStr">
+      <c r="B127" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-04</t>
         </is>
       </c>
-      <c r="C102" s="6" t="inlineStr">
+      <c r="C127" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
+      <c r="D127" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E102" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F102" s="6" t="inlineStr">
+      <c r="E127" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F127" s="6" t="inlineStr">
         <is>
           <t>local hash 473ab08fd766fe38</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="6" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B103" s="6" t="inlineStr">
+      <c r="B128" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-05</t>
         </is>
       </c>
-      <c r="C103" s="6" t="inlineStr">
+      <c r="C128" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D103" s="6" t="inlineStr">
+      <c r="D128" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E103" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F103" s="6" t="inlineStr">
+      <c r="E128" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr">
         <is>
           <t>local hash 32f952347682a67e</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="5" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
         <is>
           <t>lore_registry</t>
         </is>
       </c>
-      <c r="B104" s="5" t="inlineStr">
+      <c r="B129" s="5" t="inlineStr">
         <is>
           <t>LORE-POLICY</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C129" s="5" t="inlineStr">
         <is>
           <t>lore_policy</t>
         </is>
       </c>
-      <c r="D104" s="5" t="inlineStr">
+      <c r="D129" s="5" t="inlineStr">
         <is>
           <t>LORE</t>
         </is>
       </c>
-      <c r="E104" s="5" t="inlineStr">
+      <c r="E129" s="5" t="inlineStr">
         <is>
           <t>PUBLIC_SAFE</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr">
+      <c r="F129" s="5" t="inlineStr">
         <is>
           <t>docs/v4/resonator/LORE_AND_INTUITION_POLICY.md</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="7" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
         <is>
           <t>installer_metadata</t>
         </is>
       </c>
-      <c r="B105" s="7" t="inlineStr">
+      <c r="B130" s="7" t="inlineStr">
         <is>
           <t>REL-v4.5.0</t>
         </is>
       </c>
-      <c r="C105" s="7" t="inlineStr">
+      <c r="C130" s="7" t="inlineStr">
         <is>
           <t>release_metadata</t>
         </is>
       </c>
-      <c r="D105" s="7" t="inlineStr">
+      <c r="D130" s="7" t="inlineStr">
         <is>
           <t>DERIVED_ARITHMETIC</t>
         </is>
       </c>
-      <c r="E105" s="7" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F105" s="7" t="inlineStr">
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr">
         <is>
           <t>pyproject.toml + build</t>
         </is>
@@ -10913,57 +13026,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>evidence_class</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>privacy_class</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>provenance</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>candidate_mm</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>station_mm</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>separation_mm</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>halfwidth_mm</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>note</t>
         </is>

</xml_diff>

<commit_message>
chore(release): sync committed v4.7.1 workbook and manifest
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -30,7 +30,9 @@
     <sheet name="PMWR Recovery" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="PMWR Crystal" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="PMWR Phryll" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Workbook Guide" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="R3 Root Space" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="R3 Lanes" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Workbook Guide" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -557,6 +559,41 @@
 </table>
 </file>
 
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="R3RootSpace" displayName="R3RootSpace" ref="A1:H15" headerRowCount="1">
+  <autoFilter ref="A1:H15"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="candidates_per_second"/>
+    <tableColumn id="7" name="status"/>
+    <tableColumn id="8" name="statement"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="R3Lanes" displayName="R3Lanes" ref="A1:I5" headerRowCount="1">
+  <autoFilter ref="A1:I5"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="target_h"/>
+    <tableColumn id="7" name="region_m"/>
+    <tableColumn id="8" name="required_mass_kg"/>
+    <tableColumn id="9" name="verdict"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Specimens" displayName="Specimens" ref="A1:K2" headerRowCount="1">
   <autoFilter ref="A1:K2"/>
@@ -617,8 +654,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F130" headerRowCount="1">
-  <autoFilter ref="A1:F130"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F148" headerRowCount="1">
+  <autoFilter ref="A1:F148"/>
   <tableColumns count="6">
     <tableColumn id="1" name="table"/>
     <tableColumn id="2" name="id"/>
@@ -979,7 +1016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -996,7 +1033,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v4.7.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v4.7.1 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -1201,27 +1238,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>resonator_platform</t>
+          <t>r3_lanes</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r3_root_space</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>specimens</t>
+          <t>resonator_platform</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1231,159 +1268,179 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>specimens</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>timing_recipes</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B32" t="n">
         <v>11</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B31" s="4">
-        <f>SUM(B10:B30)</f>
-        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B33" s="4">
+        <f>SUM(B10:B32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
           <t>Evidence classes (weakest -&gt; strongest):</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>LORE</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>DERIVED_ARITHMETIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>ANALYTIC_MODEL</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>NUMERICAL_SIMULATION</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>SYNTHETIC_RUN</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>BENCH_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>INDEPENDENT_REPLICATION</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>NOT_APPLICABLE</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>METAPHOR</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>GEOMETRY_IDENTITY</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>CALIBRATED_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="18" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="18" t="inlineStr">
         <is>
           <t>ANTHROPOGENIC_STRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
         <is>
           <t>REPRESENTATION_ARTIFACT</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="20" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
         <is>
           <t>CIRCULAR_DERIVATION</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="21" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="21" t="inlineStr">
         <is>
           <t>UNEXPLAINED_INSTRUMENT_RESIDUAL</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="22" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
         <is>
           <t>REPLICATED_ANOMALY</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="23" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="23" t="inlineStr">
         <is>
           <t>PROSPECTIVE_PREDICTION</t>
         </is>
@@ -3237,7 +3294,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>4.7.0</t>
+          <t>4.7.1</t>
         </is>
       </c>
     </row>
@@ -6786,6 +6843,718 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>candidates_per_second</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>R3-ZERO-RESIDUAL-ALIASES</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>alias_audit</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>r3.root_space.zero_residual_aliases</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>4097</v>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>ROOT_ALIAS_UNRESOLVED</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>wrap(residual)=0 admits integer-cycle aliases; a zero of the wrapped residual is a candidate, never a root</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>R3-DUAL-LATTICE-ROOT</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>disambiguation</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>r3.root_space.dual_lattice_root_search</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-SYNTHETIC_HIERARCHY_ROOT</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-PHASE_AUTHORITY_ROOT</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-CALIBRATED_INSTRUMENT_ROOT</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-RECONSTRUCTED_SOURCE_STATE_ROOT</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-PHYSICAL_REFERENCE_NETWORK_ROOT</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-GAUGE_FIXED_CANONICAL_ROOT</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-HIERARCHY_ROOT_IS_VACUUM_ORIGIN</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-EIGENMODE_IS_SPACETIME_EIGENSTATE</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-PHASE_ZERO_IS_ABSOLUTE_PHASE</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-CANONICAL_REPRESENTATIVE_IS_UNIQUE_ONTOLOGY</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-REFERENCE_NETWORK_IS_PREFERRED_FRAME</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-SOURCE_ESTIMATE_IS_HISTORICAL_TRUTH</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>target_h</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>region_m</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>required_mass_kg</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>R3-METRIC-BUDGET</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>metric_source_audit</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>r3.spin_torsion.metric_actuation_verdict</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>1e-09</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>6.732954607500545e+17</v>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>REFUSED_BY_ARITHMETIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>R3-EC-TORSION-SCALE</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>spin_torsion_audit</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>r3.spin_torsion.einstein_cartan_torsion</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>UNMEASURABLE_AT_LABORATORY_SCALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>R3-HIERARCHY</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>address_hierarchy</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>r3.address.level_count</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>R3-ATLAS-STATUS</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>atlas_status</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>r3.atlas</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8824,7 +9593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12772,224 +13541,800 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="6" t="inlineStr">
-        <is>
-          <t>source_registry</t>
-        </is>
-      </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>SRC-V4X2-01</t>
-        </is>
-      </c>
-      <c r="C124" s="6" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>SOURCE_CLAIM</t>
-        </is>
-      </c>
-      <c r="E124" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F124" s="6" t="inlineStr">
-        <is>
-          <t>local hash 019435a03b3c5e9d</t>
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>R3-ZERO-RESIDUAL-ALIASES</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t>alias_audit</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr">
+        <is>
+          <t>r3.root_space.zero_residual_aliases</t>
         </is>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="6" t="inlineStr">
-        <is>
-          <t>source_registry</t>
-        </is>
-      </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>SRC-V4X2-02</t>
-        </is>
-      </c>
-      <c r="C125" s="6" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D125" s="6" t="inlineStr">
-        <is>
-          <t>SOURCE_CLAIM</t>
-        </is>
-      </c>
-      <c r="E125" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F125" s="6" t="inlineStr">
-        <is>
-          <t>local hash 7e1df086615c6bac</t>
+      <c r="A125" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
+        <is>
+          <t>R3-DUAL-LATTICE-ROOT</t>
+        </is>
+      </c>
+      <c r="C125" s="7" t="inlineStr">
+        <is>
+          <t>disambiguation</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E125" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F125" s="7" t="inlineStr">
+        <is>
+          <t>r3.root_space.dual_lattice_root_search</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="6" t="inlineStr">
-        <is>
-          <t>source_registry</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>SRC-V4X2-03</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>SOURCE_CLAIM</t>
-        </is>
-      </c>
-      <c r="E126" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr">
-        <is>
-          <t>local hash b8e387558cb0a0f0</t>
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-SYNTHETIC_HIERARCHY_ROOT</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F126" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="6" t="inlineStr">
-        <is>
-          <t>source_registry</t>
-        </is>
-      </c>
-      <c r="B127" s="6" t="inlineStr">
-        <is>
-          <t>SRC-V4X2-04</t>
-        </is>
-      </c>
-      <c r="C127" s="6" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D127" s="6" t="inlineStr">
-        <is>
-          <t>SOURCE_CLAIM</t>
-        </is>
-      </c>
-      <c r="E127" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F127" s="6" t="inlineStr">
-        <is>
-          <t>local hash 473ab08fd766fe38</t>
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-PHASE_AUTHORITY_ROOT</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E127" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="6" t="inlineStr">
-        <is>
-          <t>source_registry</t>
-        </is>
-      </c>
-      <c r="B128" s="6" t="inlineStr">
-        <is>
-          <t>SRC-V4X2-05</t>
-        </is>
-      </c>
-      <c r="C128" s="6" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D128" s="6" t="inlineStr">
-        <is>
-          <t>SOURCE_CLAIM</t>
-        </is>
-      </c>
-      <c r="E128" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F128" s="6" t="inlineStr">
-        <is>
-          <t>local hash 32f952347682a67e</t>
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-CALIBRATED_INSTRUMENT_ROOT</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F128" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="inlineStr">
-        <is>
-          <t>lore_registry</t>
-        </is>
-      </c>
-      <c r="B129" s="5" t="inlineStr">
-        <is>
-          <t>LORE-POLICY</t>
-        </is>
-      </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>lore_policy</t>
-        </is>
-      </c>
-      <c r="D129" s="5" t="inlineStr">
-        <is>
-          <t>LORE</t>
-        </is>
-      </c>
-      <c r="E129" s="5" t="inlineStr">
-        <is>
-          <t>PUBLIC_SAFE</t>
-        </is>
-      </c>
-      <c r="F129" s="5" t="inlineStr">
-        <is>
-          <t>docs/v4/resonator/LORE_AND_INTUITION_POLICY.md</t>
+      <c r="A129" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B129" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-RECONSTRUCTED_SOURCE_STATE_ROOT</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E129" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F129" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
         <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-PHYSICAL_REFERENCE_NETWORK_ROOT</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F130" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>ROOT-CLASS-GAUGE_FIXED_CANONICAL_ROOT</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t>root_class</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F131" s="7" t="inlineStr">
+        <is>
+          <t>pack core/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-HIERARCHY_ROOT_IS_VACUUM_ORIGIN</t>
+        </is>
+      </c>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E132" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F132" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-EIGENMODE_IS_SPACETIME_EIGENSTATE</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E133" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F133" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B134" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-PHASE_ZERO_IS_ABSOLUTE_PHASE</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F134" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-CANONICAL_REPRESENTATIVE_IS_UNIQUE_ONTOLOGY</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F135" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B136" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-REFERENCE_NETWORK_IS_PREFERRED_FRAME</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F136" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="7" t="inlineStr">
+        <is>
+          <t>r3_root_space</t>
+        </is>
+      </c>
+      <c r="B137" s="7" t="inlineStr">
+        <is>
+          <t>COLLAPSE-SOURCE_ESTIMATE_IS_HISTORICAL_TRUTH</t>
+        </is>
+      </c>
+      <c r="C137" s="7" t="inlineStr">
+        <is>
+          <t>forbidden_collapse</t>
+        </is>
+      </c>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E137" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F137" s="7" t="inlineStr">
+        <is>
+          <t>r3.FORBIDDEN_COLLAPSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t>r3_lanes</t>
+        </is>
+      </c>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t>R3-METRIC-BUDGET</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>metric_source_audit</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E138" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F138" s="8" t="inlineStr">
+        <is>
+          <t>r3.spin_torsion.metric_actuation_verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="8" t="inlineStr">
+        <is>
+          <t>r3_lanes</t>
+        </is>
+      </c>
+      <c r="B139" s="8" t="inlineStr">
+        <is>
+          <t>R3-EC-TORSION-SCALE</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>spin_torsion_audit</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E139" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F139" s="8" t="inlineStr">
+        <is>
+          <t>r3.spin_torsion.einstein_cartan_torsion</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t>r3_lanes</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t>R3-HIERARCHY</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t>address_hierarchy</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F140" s="7" t="inlineStr">
+        <is>
+          <t>r3.address.level_count</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t>r3_lanes</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>R3-ATLAS-STATUS</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t>atlas_status</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F141" s="7" t="inlineStr">
+        <is>
+          <t>r3.atlas</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-01</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D142" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E142" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F142" s="6" t="inlineStr">
+        <is>
+          <t>local hash 019435a03b3c5e9d</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-02</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F143" s="6" t="inlineStr">
+        <is>
+          <t>local hash 7e1df086615c6bac</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-03</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E144" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F144" s="6" t="inlineStr">
+        <is>
+          <t>local hash b8e387558cb0a0f0</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-04</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F145" s="6" t="inlineStr">
+        <is>
+          <t>local hash 473ab08fd766fe38</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-05</t>
+        </is>
+      </c>
+      <c r="C146" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F146" s="6" t="inlineStr">
+        <is>
+          <t>local hash 32f952347682a67e</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>lore_registry</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>LORE-POLICY</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>lore_policy</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>LORE</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>PUBLIC_SAFE</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>docs/v4/resonator/LORE_AND_INTUITION_POLICY.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="7" t="inlineStr">
+        <is>
           <t>installer_metadata</t>
         </is>
       </c>
-      <c r="B130" s="7" t="inlineStr">
+      <c r="B148" s="7" t="inlineStr">
         <is>
           <t>REL-v4.5.0</t>
         </is>
       </c>
-      <c r="C130" s="7" t="inlineStr">
+      <c r="C148" s="7" t="inlineStr">
         <is>
           <t>release_metadata</t>
         </is>
       </c>
-      <c r="D130" s="7" t="inlineStr">
-        <is>
-          <t>DERIVED_ARITHMETIC</t>
-        </is>
-      </c>
-      <c r="E130" s="7" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F130" s="7" t="inlineStr">
+      <c r="D148" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E148" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F148" s="7" t="inlineStr">
         <is>
           <t>pyproject.toml + build</t>
         </is>

</xml_diff>

<commit_message>
v4.8.0: release-owned artifacts committed BEFORE the tag (R04/R65)
The tag must already contain every release-owned artifact, so the
committed workbook and Windows-asset manifest are refreshed and
committed HERE, before tagging -- no post-tag sync commit.

Also fixes a determinism bug the new gate caught: the r4 canonical
rows used Python's hash() for excluded-claim record ids, which is
randomized per process (PYTHONHASHSEED), so the generated workbook
differed between runs and the gate refused a tag that was otherwise
fine. Ids are now positional. Regression test spawns two subprocesses
and asserts identical canonical ids.

1217 tests passing (CI-consistent, dist absent); qa 19/19; release
gate TAG_MAY_PROCEED.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -32,7 +32,9 @@
     <sheet name="PMWR Phryll" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="R3 Root Space" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="R3 Lanes" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Workbook Guide" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="R4 Codec" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="R4 Platforms" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Workbook Guide" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,6 +596,46 @@
 </table>
 </file>
 
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="R4Codec" displayName="R4Codec" ref="A1:J10" headerRowCount="1">
+  <autoFilter ref="A1:J10"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="identity"/>
+    <tableColumn id="7" name="keys_checked"/>
+    <tableColumn id="8" name="roundtrip_ok"/>
+    <tableColumn id="9" name="is_compression"/>
+    <tableColumn id="10" name="note"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="R4Platforms" displayName="R4Platforms" ref="A1:L17" headerRowCount="1">
+  <autoFilter ref="A1:L17"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="type"/>
+    <tableColumn id="7" name="native_levels"/>
+    <tableColumn id="8" name="orthogonal"/>
+    <tableColumn id="9" name="coherent"/>
+    <tableColumn id="10" name="selectable"/>
+    <tableColumn id="11" name="open_gates"/>
+    <tableColumn id="12" name="limitations"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Specimens" displayName="Specimens" ref="A1:K2" headerRowCount="1">
   <autoFilter ref="A1:K2"/>
@@ -654,8 +696,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F148" headerRowCount="1">
-  <autoFilter ref="A1:F148"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F173" headerRowCount="1">
+  <autoFilter ref="A1:F173"/>
   <tableColumns count="6">
     <tableColumn id="1" name="table"/>
     <tableColumn id="2" name="id"/>
@@ -1016,7 +1058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1033,7 +1075,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v4.7.1 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v4.8.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -1258,27 +1300,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>resonator_platform</t>
+          <t>r4_codec</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r4_platforms</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>specimens</t>
+          <t>resonator_platform</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1288,159 +1330,179 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>specimens</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>timing_recipes</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B34" t="n">
         <v>11</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B33" s="4">
-        <f>SUM(B10:B32)</f>
-        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B35" s="4">
+        <f>SUM(B10:B34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
           <t>Evidence classes (weakest -&gt; strongest):</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>LORE</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>DERIVED_ARITHMETIC</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>ANALYTIC_MODEL</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>NUMERICAL_SIMULATION</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>SYNTHETIC_RUN</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>BENCH_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>INDEPENDENT_REPLICATION</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>NOT_APPLICABLE</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>METAPHOR</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>GEOMETRY_IDENTITY</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>CALIBRATED_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="18" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>ANTHROPOGENIC_STRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="19" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>REPRESENTATION_ARTIFACT</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="20" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr">
         <is>
           <t>CIRCULAR_DERIVATION</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="21" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="21" t="inlineStr">
         <is>
           <t>UNEXPLAINED_INSTRUMENT_RESIDUAL</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>REPLICATED_ANOMALY</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="23" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="23" t="inlineStr">
         <is>
           <t>PROSPECTIVE_PREDICTION</t>
         </is>
@@ -3294,7 +3356,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>4.7.1</t>
+          <t>4.8.0</t>
         </is>
       </c>
     </row>
@@ -7555,6 +7617,1120 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>keys_checked</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>roundtrip_ok</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>is_compression</t>
+        </is>
+      </c>
+      <c r="J1" s="24" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>R4-RADIX-BRIDGE</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>radix_identity</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>r4.radix.exhaustive_roundtrip</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>4096 = 8^4 = 4^6 = 2^12 ; 64 = 8^2 = 4^3 = 2^6</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>4096</v>
+      </c>
+      <c r="H2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>exact radix conversion contributes ZERO compression</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>R4-TETRA-CODEBOOK</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>codebook_geometry</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>r4.quantizer.codebook_geometry</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>four directions at -1/3 overlap are NOT an orthogonal basis; they cannot hold two bits in one spin-1/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-SMOOTH_FIELD</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="n"/>
+      <c r="J4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-PIECEWISE_CONSTANT</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-SPARSE_EVENTS</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-PHASE_RAMP</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-RANDOM_UNIFORM</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-RANDOM_GAUSSIAN</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>R4-NEGATIVE-CONTROL-GATE</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>campaign_gate</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="24" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>native_levels</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>orthogonal</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>coherent</t>
+        </is>
+      </c>
+      <c r="J1" s="24" t="inlineStr">
+        <is>
+          <t>selectable</t>
+        </is>
+      </c>
+      <c r="K1" s="24" t="inlineStr">
+        <is>
+          <t>open_gates</t>
+        </is>
+      </c>
+      <c r="L1" s="24" t="inlineStr">
+        <is>
+          <t>limitations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>SIC_V_SI_SPIN_3_2</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>SPIN_THREE_HALVES</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>full four-level discrimination is nontrivial: optical readout commonly distinguishes |m_s|=1/2 from |m_s|=3/2 PAIRS rather than all four levels, so sign resolution needs extra cont</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>DIAMOND_NV_PLUS_N15</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>TWO_COUPLED_SPIN_HALF</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>four states come from TWO spins, not one four-level system; addressing density is limited by optical diffraction unless super-resolution is used</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>CLASSICAL_FOUR_DOMAIN</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>FOUR_CLASSICAL_DOMAINS</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>NOT coherent spin memory. Perfectly good for quaternary symbol storage; it tests the codec, not the spin hypothesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>SPIN_HALF_TETRAHEDRAL</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>SPIN_HALF_FOUR_DIRECTIONS</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>REFUSED as memory: a spin-1/2 has a 2-dimensional Hilbert space. Four non-orthogonal directions (overlap -1/3) cannot be deterministically distinguished, so they do not store two b</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>QUARTZ_DEFECT</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>QUARTZ_DEFECT_PLATFORM</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>BLOCKED: no identified defect with a demonstrated write/read/reset chain in this programme's specimen. The source narrative motivates the lane; it does not qualify the platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>R4-PLATFORM-DECISION</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>decision_matrix</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.decision_matrix</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>R4-BENCH-READINESS</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>honest_stop</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>r4.bench.bench_readiness</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-00</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="n"/>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-01</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+      <c r="I10" s="13" t="n"/>
+      <c r="J10" s="13" t="n"/>
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-02</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+      <c r="H11" s="13" t="n"/>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="n"/>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="13" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-03</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="13" t="n"/>
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-04</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-05</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="13" t="n"/>
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-06</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="13" t="n"/>
+      <c r="K15" s="13" t="n"/>
+      <c r="L15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-07</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="13" t="n"/>
+      <c r="K16" s="13" t="n"/>
+      <c r="L16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-08</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="n"/>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="13" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9593,7 +10769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -14117,224 +15293,1024 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="6" t="inlineStr">
+      <c r="A142" s="7" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
+        <is>
+          <t>R4-RADIX-BRIDGE</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>radix_identity</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F142" s="7" t="inlineStr">
+        <is>
+          <t>r4.radix.exhaustive_roundtrip</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>R4-TETRA-CODEBOOK</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t>codebook_geometry</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F143" s="7" t="inlineStr">
+        <is>
+          <t>r4.quantizer.codebook_geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-SMOOTH_FIELD</t>
+        </is>
+      </c>
+      <c r="C144" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E144" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F144" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-PIECEWISE_CONSTANT</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-SPARSE_EVENTS</t>
+        </is>
+      </c>
+      <c r="C146" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E146" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F146" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-PHASE_RAMP</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F147" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-RANDOM_UNIFORM</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E148" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F148" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>R4-BENCH-RANDOM_GAUSSIAN</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>rate_distortion</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="9" t="inlineStr">
+        <is>
+          <t>r4_codec</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>R4-NEGATIVE-CONTROL-GATE</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>campaign_gate</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>NUMERICAL_SIMULATION</t>
+        </is>
+      </c>
+      <c r="E150" s="9" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F150" s="9" t="inlineStr">
+        <is>
+          <t>r4.benchmark.full_campaign</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B151" s="8" t="inlineStr">
+        <is>
+          <t>SIC_V_SI_SPIN_3_2</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E151" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F151" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>DIAMOND_NV_PLUS_N15</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="D152" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E152" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F152" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B153" s="8" t="inlineStr">
+        <is>
+          <t>CLASSICAL_FOUR_DOMAIN</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E153" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F153" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>SPIN_HALF_TETRAHEDRAL</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="D154" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E154" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F154" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B155" s="8" t="inlineStr">
+        <is>
+          <t>QUARTZ_DEFECT</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>four_state_platform</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E155" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F155" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.REGISTRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>R4-PLATFORM-DECISION</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>decision_matrix</t>
+        </is>
+      </c>
+      <c r="D156" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E156" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F156" s="8" t="inlineStr">
+        <is>
+          <t>r4.platforms.decision_matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="8" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B157" s="8" t="inlineStr">
+        <is>
+          <t>R4-BENCH-READINESS</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t>honest_stop</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="inlineStr">
+        <is>
+          <t>ANALYTIC_MODEL</t>
+        </is>
+      </c>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F157" s="8" t="inlineStr">
+        <is>
+          <t>r4.bench.bench_readiness</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B158" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-00</t>
+        </is>
+      </c>
+      <c r="C158" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D158" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E158" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F158" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B159" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-01</t>
+        </is>
+      </c>
+      <c r="C159" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D159" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E159" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F159" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B160" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-02</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D160" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E160" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F160" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B161" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-03</t>
+        </is>
+      </c>
+      <c r="C161" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D161" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E161" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F161" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B162" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-04</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D162" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E162" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F162" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B163" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-05</t>
+        </is>
+      </c>
+      <c r="C163" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D163" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E163" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F163" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B164" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-06</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D164" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E164" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F164" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B165" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-07</t>
+        </is>
+      </c>
+      <c r="C165" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D165" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E165" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F165" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="13" t="inlineStr">
+        <is>
+          <t>r4_platforms</t>
+        </is>
+      </c>
+      <c r="B166" s="13" t="inlineStr">
+        <is>
+          <t>R4-EXCLUDED-08</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="inlineStr">
+        <is>
+          <t>excluded_claim</t>
+        </is>
+      </c>
+      <c r="D166" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E166" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F166" s="13" t="inlineStr">
+        <is>
+          <t>r4.EXCLUDED_CLAIMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B142" s="6" t="inlineStr">
+      <c r="B167" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-01</t>
         </is>
       </c>
-      <c r="C142" s="6" t="inlineStr">
+      <c r="C167" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D142" s="6" t="inlineStr">
+      <c r="D167" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E142" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F142" s="6" t="inlineStr">
+      <c r="E167" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F167" s="6" t="inlineStr">
         <is>
           <t>local hash 019435a03b3c5e9d</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="6" t="inlineStr">
+    <row r="168">
+      <c r="A168" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B143" s="6" t="inlineStr">
+      <c r="B168" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-02</t>
         </is>
       </c>
-      <c r="C143" s="6" t="inlineStr">
+      <c r="C168" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D143" s="6" t="inlineStr">
+      <c r="D168" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E143" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F143" s="6" t="inlineStr">
+      <c r="E168" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F168" s="6" t="inlineStr">
         <is>
           <t>local hash 7e1df086615c6bac</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="6" t="inlineStr">
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B144" s="6" t="inlineStr">
+      <c r="B169" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-03</t>
         </is>
       </c>
-      <c r="C144" s="6" t="inlineStr">
+      <c r="C169" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D144" s="6" t="inlineStr">
+      <c r="D169" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E144" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F144" s="6" t="inlineStr">
+      <c r="E169" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F169" s="6" t="inlineStr">
         <is>
           <t>local hash b8e387558cb0a0f0</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="6" t="inlineStr">
+    <row r="170">
+      <c r="A170" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B145" s="6" t="inlineStr">
+      <c r="B170" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-04</t>
         </is>
       </c>
-      <c r="C145" s="6" t="inlineStr">
+      <c r="C170" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D145" s="6" t="inlineStr">
+      <c r="D170" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E145" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F145" s="6" t="inlineStr">
+      <c r="E170" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F170" s="6" t="inlineStr">
         <is>
           <t>local hash 473ab08fd766fe38</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="6" t="inlineStr">
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
         <is>
           <t>source_registry</t>
         </is>
       </c>
-      <c r="B146" s="6" t="inlineStr">
+      <c r="B171" s="6" t="inlineStr">
         <is>
           <t>SRC-V4X2-05</t>
         </is>
       </c>
-      <c r="C146" s="6" t="inlineStr">
+      <c r="C171" s="6" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="D146" s="6" t="inlineStr">
+      <c r="D171" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
-      <c r="E146" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F146" s="6" t="inlineStr">
+      <c r="E171" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F171" s="6" t="inlineStr">
         <is>
           <t>local hash 32f952347682a67e</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="5" t="inlineStr">
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
         <is>
           <t>lore_registry</t>
         </is>
       </c>
-      <c r="B147" s="5" t="inlineStr">
+      <c r="B172" s="5" t="inlineStr">
         <is>
           <t>LORE-POLICY</t>
         </is>
       </c>
-      <c r="C147" s="5" t="inlineStr">
+      <c r="C172" s="5" t="inlineStr">
         <is>
           <t>lore_policy</t>
         </is>
       </c>
-      <c r="D147" s="5" t="inlineStr">
+      <c r="D172" s="5" t="inlineStr">
         <is>
           <t>LORE</t>
         </is>
       </c>
-      <c r="E147" s="5" t="inlineStr">
+      <c r="E172" s="5" t="inlineStr">
         <is>
           <t>PUBLIC_SAFE</t>
         </is>
       </c>
-      <c r="F147" s="5" t="inlineStr">
+      <c r="F172" s="5" t="inlineStr">
         <is>
           <t>docs/v4/resonator/LORE_AND_INTUITION_POLICY.md</t>
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="7" t="inlineStr">
+    <row r="173">
+      <c r="A173" s="7" t="inlineStr">
         <is>
           <t>installer_metadata</t>
         </is>
       </c>
-      <c r="B148" s="7" t="inlineStr">
+      <c r="B173" s="7" t="inlineStr">
         <is>
           <t>REL-v4.5.0</t>
         </is>
       </c>
-      <c r="C148" s="7" t="inlineStr">
+      <c r="C173" s="7" t="inlineStr">
         <is>
           <t>release_metadata</t>
         </is>
       </c>
-      <c r="D148" s="7" t="inlineStr">
+      <c r="D173" s="7" t="inlineStr">
         <is>
           <t>DERIVED_ARITHMETIC</t>
         </is>
       </c>
-      <c r="E148" s="7" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F148" s="7" t="inlineStr">
+      <c r="E173" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F173" s="7" t="inlineStr">
         <is>
           <t>pyproject.toml + build</t>
         </is>

</xml_diff>

<commit_message>
v5.0.0: R7 release artifacts and metadata
Version bumped to 5.0.0 with release notes, CHANGELOG entry and
workbook at 39 sheets. Release gate TAG_MAY_PROCEED, QA audit 19/19.

The documented test count is 2166, and arriving at it needed care.
The count guards are self-referential: while the documented figure
disagrees with reality, three version/count tests fail, so a refresh
run measures 2163 and would pin that -- a number that becomes wrong
the moment it is written down, because writing it makes the guards
pass. 2166 is the fixed point: with the docs consistent the guards
pass and the total is 2166. Verified by a clean run rather than
assumed, and the reasoning is recorded in RELEASE_METADATA.json so
the next bump does not rediscover it.

Publication path remains PRIVATE_RC. This release is created on a
PRIVATE repository and publishes nothing; it exists to preserve
artifacts for a later decision.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1,47 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frequency Keys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harmonic Relations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specimens" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Estimates" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timing Recipes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypotheses" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Ledger" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eye Results" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resonator Platform" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware BOM" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiment Queue" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrections" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Registry" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lore Registry" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Installer Metadata" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSCP Candidates" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSCP Tetrahedron" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSCP Spacetime" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CSCP Experiments" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PMWR Recovery" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PMWR Crystal" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PMWR Phryll" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R3 Root Space" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R3 Lanes" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R4 Codec" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R4 Platforms" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Claims" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Apparatus" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Witness" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Mailbox" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Grid" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Instruments" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R6 Governance" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook Guide" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Frequency Keys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Harmonic Relations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Specimens" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mode Estimates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Timing Recipes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Hypotheses" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Evidence Ledger" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Eye Results" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Resonator Platform" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Hardware BOM" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Experiment Queue" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Corrections" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Source Registry" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Lore Registry" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Installer Metadata" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="CSCP Candidates" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="CSCP Tetrahedron" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="CSCP Spacetime" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="CSCP Experiments" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="PMWR Recovery" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="PMWR Crystal" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="PMWR Phryll" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="R3 Root Space" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="R3 Lanes" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="R4 Codec" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="R4 Platforms" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="R6 Claims" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="R6 Apparatus" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="R6 Witness" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="R6 Mailbox" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="R6 Grid" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="R6 Instruments" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="R6 Governance" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="R7 CW" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="R7 Gravity" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="R7 Clock Link" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="R7 Governance" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="Workbook Guide" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -953,6 +957,132 @@
 </table>
 </file>
 
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="R7CW" displayName="R7CW" ref="A1:AC9" headerRowCount="1">
+  <autoFilter ref="A1:AC9"/>
+  <tableColumns count="29">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="claim"/>
+    <tableColumn id="7" name="status"/>
+    <tableColumn id="8" name="forced_common_bits"/>
+    <tableColumn id="9" name="observed_common_bits"/>
+    <tableColumn id="10" name="informative_bits"/>
+    <tableColumn id="11" name="header_is_forced_by_span"/>
+    <tableColumn id="12" name="null_3x12_p_both"/>
+    <tableColumn id="13" name="null_6x6_p_both"/>
+    <tableColumn id="14" name="verdict"/>
+    <tableColumn id="15" name="ceiling"/>
+    <tableColumn id="16" name="source_string"/>
+    <tableColumn id="17" name="value"/>
+    <tableColumn id="18" name="bit_length"/>
+    <tableColumn id="19" name="header_3x12"/>
+    <tableColumn id="20" name="field1_3x12"/>
+    <tableColumn id="21" name="field2_3x12"/>
+    <tableColumn id="22" name="field3_3x12"/>
+    <tableColumn id="23" name="note"/>
+    <tableColumn id="24" name="parse"/>
+    <tableColumn id="25" name="header_bits"/>
+    <tableColumn id="26" name="field_bits"/>
+    <tableColumn id="27" name="n_fields"/>
+    <tableColumn id="28" name="digest"/>
+    <tableColumn id="29" name="semantics_declared"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="R7Gravity" displayName="R7Gravity" ref="A1:U6" headerRowCount="1">
+  <autoFilter ref="A1:U6"/>
+  <tableColumns count="21">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="configuration"/>
+    <tableColumn id="7" name="total_energy_j"/>
+    <tableColumn id="8" name="equivalent_mass_kg"/>
+    <tableColumn id="9" name="predicted_fractional_shift"/>
+    <tableColumn id="10" name="predicted_acceleration_ms2"/>
+    <tableColumn id="11" name="clock_gap_decades"/>
+    <tableColumn id="12" name="acceleration_gap_decades"/>
+    <tableColumn id="13" name="status"/>
+    <tableColumn id="14" name="note"/>
+    <tableColumn id="15" name="all_refused"/>
+    <tableColumn id="16" name="configurations_refused"/>
+    <tableColumn id="17" name="reference_1mm_height_shift"/>
+    <tableColumn id="18" name="ratio_1mm_lift_over_best_apparatus"/>
+    <tableColumn id="19" name="verdict"/>
+    <tableColumn id="20" name="consequence"/>
+    <tableColumn id="21" name="what_this_does_not_say"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="R7ClockLink" displayName="R7ClockLink" ref="A1:S18" headerRowCount="1">
+  <autoFilter ref="A1:S18"/>
+  <tableColumns count="19">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="oscillator"/>
+    <tableColumn id="7" name="link"/>
+    <tableColumn id="8" name="target_height_m"/>
+    <tableColumn id="9" name="target_fractional"/>
+    <tableColumn id="10" name="combined_floor"/>
+    <tableColumn id="11" name="limiter"/>
+    <tableColumn id="12" name="resolvable"/>
+    <tableColumn id="13" name="tau_required_years"/>
+    <tableColumn id="14" name="status"/>
+    <tableColumn id="15" name="consumer_quartz_unresolvable"/>
+    <tableColumn id="16" name="link_limited_pairings"/>
+    <tableColumn id="17" name="claim_ceiling"/>
+    <tableColumn id="18" name="bottleneck_note"/>
+    <tableColumn id="19" name="why_run_it_anyway"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="R7Governance" displayName="R7Governance" ref="A1:U6" headerRowCount="1">
+  <autoFilter ref="A1:U6"/>
+  <tableColumns count="21">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="kind"/>
+    <tableColumn id="3" name="evidence_class"/>
+    <tableColumn id="4" name="privacy_class"/>
+    <tableColumn id="5" name="provenance"/>
+    <tableColumn id="6" name="path"/>
+    <tableColumn id="7" name="signed_by"/>
+    <tableColumn id="8" name="signed_at"/>
+    <tableColumn id="9" name="digest"/>
+    <tableColumn id="10" name="complete"/>
+    <tableColumn id="11" name="reversible"/>
+    <tableColumn id="12" name="authorized_to_publish"/>
+    <tableColumn id="13" name="status"/>
+    <tableColumn id="14" name="note"/>
+    <tableColumn id="15" name="provides"/>
+    <tableColumn id="16" name="does_not_provide"/>
+    <tableColumn id="17" name="why_it_matters"/>
+    <tableColumn id="18" name="preserves_patent_rights"/>
+    <tableColumn id="19" name="creates_public_prior_art"/>
+    <tableColumn id="20" name="forecloses"/>
+    <tableColumn id="21" name="cost"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TimingRecipes" displayName="TimingRecipes" ref="A1:K12" headerRowCount="1">
   <autoFilter ref="A1:K12"/>
@@ -993,8 +1123,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F237" headerRowCount="1">
-  <autoFilter ref="A1:F237"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EvidenceLedger" displayName="EvidenceLedger" ref="A1:F272" headerRowCount="1">
+  <autoFilter ref="A1:F272"/>
   <tableColumns count="6">
     <tableColumn id="1" name="table"/>
     <tableColumn id="2" name="id"/>
@@ -1358,7 +1488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1375,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v4.9.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.0.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -1690,210 +1820,250 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>resonator_platform</t>
+          <t>r7_clocklink</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r7_cw</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>specimens</t>
+          <t>r7_governance</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>r7_gravity</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>resonator_platform</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>specimens</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>timing_recipes</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B45" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B42" s="4">
-        <f>SUM(B10:B41)</f>
+      <c r="B46" s="4">
+        <f>SUM(B10:B45)</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Evidence classes (weakest -&gt; strongest):</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>LORE</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>SOURCE_CLAIM</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>DERIVED_ARITHMETIC</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>ANALYTIC_MODEL</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="9" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>NUMERICAL_SIMULATION</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t>SYNTHETIC_RUN</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>BENCH_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t>INDEPENDENT_REPLICATION</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="13" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>UNSUPPORTED</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>NOT_APPLICABLE</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="15" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>METAPHOR</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="16" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>GEOMETRY_IDENTITY</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>CALIBRATED_MEASUREMENT</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="18" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
         <is>
           <t>ANTHROPOGENIC_STRUCTURE</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="19" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="19" t="inlineStr">
         <is>
           <t>REPRESENTATION_ARTIFACT</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="20" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="20" t="inlineStr">
         <is>
           <t>CIRCULAR_DERIVATION</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="21" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="21" t="inlineStr">
         <is>
           <t>UNEXPLAINED_INSTRUMENT_RESIDUAL</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="22" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>REPLICATED_ANOMALY</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="23" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="23" t="inlineStr">
         <is>
           <t>PROSPECTIVE_PREDICTION</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="24" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="24" t="inlineStr">
         <is>
           <t>OPERATIONAL_HYPOTHESIS</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="25" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="25" t="inlineStr">
         <is>
           <t>ORDINARY_CHANNEL_RESULT</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="26" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="26" t="inlineStr">
         <is>
           <t>CANDIDATE_NEW_MECHANISM</t>
         </is>
@@ -3823,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>4.9.0</t>
+          <t>5.0.0</t>
         </is>
       </c>
     </row>
@@ -16125,6 +16295,2969 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:AC9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="60" customWidth="1" min="23" max="23"/>
+    <col width="19" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="60" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>forced_common_bits</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>observed_common_bits</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>informative_bits</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>header_is_forced_by_span</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>null_3x12_p_both</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>null_6x6_p_both</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="O1" s="27" t="inlineStr">
+        <is>
+          <t>ceiling</t>
+        </is>
+      </c>
+      <c r="P1" s="27" t="inlineStr">
+        <is>
+          <t>source_string</t>
+        </is>
+      </c>
+      <c r="Q1" s="27" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="R1" s="27" t="inlineStr">
+        <is>
+          <t>bit_length</t>
+        </is>
+      </c>
+      <c r="S1" s="27" t="inlineStr">
+        <is>
+          <t>header_3x12</t>
+        </is>
+      </c>
+      <c r="T1" s="27" t="inlineStr">
+        <is>
+          <t>field1_3x12</t>
+        </is>
+      </c>
+      <c r="U1" s="27" t="inlineStr">
+        <is>
+          <t>field2_3x12</t>
+        </is>
+      </c>
+      <c r="V1" s="27" t="inlineStr">
+        <is>
+          <t>field3_3x12</t>
+        </is>
+      </c>
+      <c r="W1" s="27" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="X1" s="27" t="inlineStr">
+        <is>
+          <t>parse</t>
+        </is>
+      </c>
+      <c r="Y1" s="27" t="inlineStr">
+        <is>
+          <t>header_bits</t>
+        </is>
+      </c>
+      <c r="Z1" s="27" t="inlineStr">
+        <is>
+          <t>field_bits</t>
+        </is>
+      </c>
+      <c r="AA1" s="27" t="inlineStr">
+        <is>
+          <t>n_fields</t>
+        </is>
+      </c>
+      <c r="AB1" s="27" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="AC1" s="27" t="inlineStr">
+        <is>
+          <t>semantics_declared</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>R7-CW-PARSE-NULL</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>parse_null</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>r7.cw.status_report</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>the five CW strings encode a header plus 4096-state fields</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>CW_PARSE_RETROSPECTIVE</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>The shared header and shared leading field are forced by the values' span, not by any encoding. Random integers drawn from the same interval reproduce the same 'structure' at a rate of 1.000. The observation is compatible with a protocol and is equally compatible with five arbitrary numbers that happen to be close together, so it discriminates between them not at all.</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>CW_PARSE_RETROSPECTIVE</t>
+        </is>
+      </c>
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="n"/>
+      <c r="U2" s="7" t="n"/>
+      <c r="V2" s="7" t="n"/>
+      <c r="W2" s="7" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
+      <c r="Z2" s="7" t="n"/>
+      <c r="AA2" s="7" t="n"/>
+      <c r="AB2" s="7" t="n"/>
+      <c r="AC2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>R7-CW-VECTOR-00</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>source_vector</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>JH corpus CW vector strings</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+      <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="n"/>
+      <c r="M3" s="6" t="n"/>
+      <c r="N3" s="6" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="inlineStr">
+        <is>
+          <t>162875493612</t>
+        </is>
+      </c>
+      <c r="Q3" s="6" t="n">
+        <v>162875493612</v>
+      </c>
+      <c r="R3" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T3" s="6" t="n">
+        <v>1516</v>
+      </c>
+      <c r="U3" s="6" t="n">
+        <v>556</v>
+      </c>
+      <c r="V3" s="6" t="n">
+        <v>3308</v>
+      </c>
+      <c r="W3" s="6" t="inlineStr">
+        <is>
+          <t>header and field1 lie inside the 15 leading bits forced identical by the interval; only fields 2 and 3 carry any variation</t>
+        </is>
+      </c>
+      <c r="X3" s="6" t="n"/>
+      <c r="Y3" s="6" t="n"/>
+      <c r="Z3" s="6" t="n"/>
+      <c r="AA3" s="6" t="n"/>
+      <c r="AB3" s="6" t="n"/>
+      <c r="AC3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>R7-CW-VECTOR-01</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>source_vector</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>JH corpus CW vector strings</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="n"/>
+      <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>162875432975</t>
+        </is>
+      </c>
+      <c r="Q4" s="6" t="n">
+        <v>162875432975</v>
+      </c>
+      <c r="R4" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T4" s="6" t="n">
+        <v>1516</v>
+      </c>
+      <c r="U4" s="6" t="n">
+        <v>542</v>
+      </c>
+      <c r="V4" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="W4" s="6" t="inlineStr">
+        <is>
+          <t>header and field1 lie inside the 15 leading bits forced identical by the interval; only fields 2 and 3 carry any variation</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="n"/>
+      <c r="Y4" s="6" t="n"/>
+      <c r="Z4" s="6" t="n"/>
+      <c r="AA4" s="6" t="n"/>
+      <c r="AB4" s="6" t="n"/>
+      <c r="AC4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>R7-CW-VECTOR-02</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>source_vector</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>JH corpus CW vector strings</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="n"/>
+      <c r="M5" s="6" t="n"/>
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>162877542769</t>
+        </is>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>162877542769</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>1516</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>1057</v>
+      </c>
+      <c r="V5" s="6" t="n">
+        <v>369</v>
+      </c>
+      <c r="W5" s="6" t="inlineStr">
+        <is>
+          <t>header and field1 lie inside the 15 leading bits forced identical by the interval; only fields 2 and 3 carry any variation</t>
+        </is>
+      </c>
+      <c r="X5" s="6" t="n"/>
+      <c r="Y5" s="6" t="n"/>
+      <c r="Z5" s="6" t="n"/>
+      <c r="AA5" s="6" t="n"/>
+      <c r="AB5" s="6" t="n"/>
+      <c r="AC5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>R7-CW-VECTOR-03</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>source_vector</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>JH corpus CW vector strings</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="6" t="n"/>
+      <c r="N6" s="6" t="n"/>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>162875439275</t>
+        </is>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>162875439275</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>1516</v>
+      </c>
+      <c r="U6" s="6" t="n">
+        <v>543</v>
+      </c>
+      <c r="V6" s="6" t="n">
+        <v>2219</v>
+      </c>
+      <c r="W6" s="6" t="inlineStr">
+        <is>
+          <t>header and field1 lie inside the 15 leading bits forced identical by the interval; only fields 2 and 3 carry any variation</t>
+        </is>
+      </c>
+      <c r="X6" s="6" t="n"/>
+      <c r="Y6" s="6" t="n"/>
+      <c r="Z6" s="6" t="n"/>
+      <c r="AA6" s="6" t="n"/>
+      <c r="AB6" s="6" t="n"/>
+      <c r="AC6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>R7-CW-VECTOR-04</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>source_vector</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>JH corpus CW vector strings</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="n"/>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>162875439285</t>
+        </is>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>162875439285</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>1516</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>543</v>
+      </c>
+      <c r="V7" s="6" t="n">
+        <v>2229</v>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t>header and field1 lie inside the 15 leading bits forced identical by the interval; only fields 2 and 3 carry any variation</t>
+        </is>
+      </c>
+      <c r="X7" s="6" t="n"/>
+      <c r="Y7" s="6" t="n"/>
+      <c r="Z7" s="6" t="n"/>
+      <c r="AA7" s="6" t="n"/>
+      <c r="AB7" s="6" t="n"/>
+      <c r="AC7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>R7-CW-DECODER-HEADER2_PLUS_3X12</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>frozen_decoder</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>r7.cw.FROZEN_DECODERS</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="inlineStr">
+        <is>
+          <t>frozen by digest so future vectors test it prospectively; reassignment raises</t>
+        </is>
+      </c>
+      <c r="X8" s="7" t="inlineStr">
+        <is>
+          <t>HEADER2_PLUS_3X12</t>
+        </is>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z8" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB8" s="7" t="inlineStr">
+        <is>
+          <t>5abb080761489f51851367453beafa037c8d04bb5141d55922909ef26a365b71</t>
+        </is>
+      </c>
+      <c r="AC8" s="7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>R7-CW-DECODER-HEADER2_PLUS_6X6</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>frozen_decoder</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>r7.cw.FROZEN_DECODERS</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="n"/>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
+      <c r="Q9" s="7" t="n"/>
+      <c r="R9" s="7" t="n"/>
+      <c r="S9" s="7" t="n"/>
+      <c r="T9" s="7" t="n"/>
+      <c r="U9" s="7" t="n"/>
+      <c r="V9" s="7" t="n"/>
+      <c r="W9" s="7" t="inlineStr">
+        <is>
+          <t>frozen by digest so future vectors test it prospectively; reassignment raises</t>
+        </is>
+      </c>
+      <c r="X9" s="7" t="inlineStr">
+        <is>
+          <t>HEADER2_PLUS_6X6</t>
+        </is>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z9" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA9" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB9" s="7" t="inlineStr">
+        <is>
+          <t>8db7a8c3afe61501050906e228f41484aeb87d159d3c157a446e34b1e4165c09</t>
+        </is>
+      </c>
+      <c r="AC9" s="7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
+    <col width="60" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>configuration</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>total_energy_j</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>equivalent_mass_kg</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>predicted_fractional_shift</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>predicted_acceleration_ms2</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>clock_gap_decades</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>acceleration_gap_decades</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="O1" s="27" t="inlineStr">
+        <is>
+          <t>all_refused</t>
+        </is>
+      </c>
+      <c r="P1" s="27" t="inlineStr">
+        <is>
+          <t>configurations_refused</t>
+        </is>
+      </c>
+      <c r="Q1" s="27" t="inlineStr">
+        <is>
+          <t>reference_1mm_height_shift</t>
+        </is>
+      </c>
+      <c r="R1" s="27" t="inlineStr">
+        <is>
+          <t>ratio_1mm_lift_over_best_apparatus</t>
+        </is>
+      </c>
+      <c r="S1" s="27" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="T1" s="27" t="inlineStr">
+        <is>
+          <t>consequence</t>
+        </is>
+      </c>
+      <c r="U1" s="27" t="inlineStr">
+        <is>
+          <t>what_this_does_not_say</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-HANDHELD_CRYSTAL</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>HANDHELD_CRYSTAL</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1.001e-06</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>1.113762706109672e-23</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>8.270980357337734e-50</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>7.433586429387782e-32</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>30.08244301057463</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>20.12880160471878</v>
+      </c>
+      <c r="M2" s="7" t="inlineStr">
+        <is>
+          <t>REFUSED_BY_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>the predicted effect is 20.1 orders of magnitude below the best instrument that exists. Averaging reduces white noise as sqrt(t), so closing 20.1 decades would need about 10^40 seconds of integration -- unreachable regardless of patience or funding.</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="n"/>
+      <c r="U2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-BENCH_COIL_DRIVE</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>BENCH_COIL_DRIVE</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>19.001</v>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>2.114146371507481e-16</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>1.569998978719024e-42</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>1.411044712735237e-24</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>22.8041006300983</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>12.85045922424245</v>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>REFUSED_BY_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>the predicted effect is 12.9 orders of magnitude below the best instrument that exists. Averaging reduces white noise as sqrt(t), so closing 12.9 decades would need about 10^26 seconds of integration -- unreachable regardless of patience or funding.</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="7" t="n"/>
+      <c r="Q3" s="7" t="n"/>
+      <c r="R3" s="7" t="n"/>
+      <c r="S3" s="7" t="n"/>
+      <c r="T3" s="7" t="n"/>
+      <c r="U3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-HIGH_POWER_PULSE</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>HIGH_POWER_PULSE</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2900</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>3.226685162555494e-14</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>2.396188115512431e-40</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>2.153586478044412e-22</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>20.62047909015499</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>10.66683768429914</v>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>REFUSED_BY_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>the predicted effect is 10.7 orders of magnitude below the best instrument that exists. Averaging reduces white noise as sqrt(t), so closing 10.7 decades would need about 10^21 seconds of integration -- unreachable regardless of patience or funding.</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="7" t="n"/>
+      <c r="Q4" s="7" t="n"/>
+      <c r="R4" s="7" t="n"/>
+      <c r="S4" s="7" t="n"/>
+      <c r="T4" s="7" t="n"/>
+      <c r="U4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-ABSURD_UPPER_BOUND</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>ABSURD_UPPER_BOUND</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>2.225300112107237e-11</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>1.652543527939607e-37</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>1.485232053823733e-19</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>17.78184709238997</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>7.828205686534115</v>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>REFUSED_BY_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>the predicted effect is 7.8 orders of magnitude below the best instrument that exists. Averaging reduces white noise as sqrt(t), so closing 7.8 decades would need about 10^16 seconds of integration -- unreachable regardless of patience or funding.</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
+      <c r="Q5" s="7" t="n"/>
+      <c r="R5" s="7" t="n"/>
+      <c r="S5" s="7" t="n"/>
+      <c r="T5" s="7" t="n"/>
+      <c r="U5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-VERDICT</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>gravity_verdict</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.full_assessment</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>HANDHELD_CRYSTAL; BENCH_COIL_DRIVE; HIGH_POWER_PULSE; ABSURD_UPPER_BOUND</t>
+        </is>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v>1.091136967219822e-19</v>
+      </c>
+      <c r="R6" s="7" t="n">
+        <v>6.602772930164522e+17</v>
+      </c>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>Every configuration, including a deliberately absurd one-megajoule upper bound far beyond anything this programme could build or safely operate, is refused by arithmetic. Raising a clock by one millimetre against Earth's field produces a larger fractional shift than the entire apparatus does by 6.6e+17 times. The apparatus is not competing with a subtle effect; it is competing with the floor of the building.</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>No metric-actuation claim can be tested by this apparatus, at any energy it could reach, with any instrument that exists. This is the strongest form of negative result the programme can produce: it does not depend on the crystal, the geometry, the drive pattern or the source corpus being right or wrong.</t>
+        </is>
+      </c>
+      <c r="U6" s="7" t="inlineStr">
+        <is>
+          <t>It does not say relativity is untestable at bench scale. Optical clocks resolve centimetre height differences routinely. It says the apparatus's OWN stress-energy is irrelevant, so any real experiment here measures Earth's field, not the device's.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="47" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>oscillator</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>target_height_m</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>target_fractional</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>combined_floor</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>limiter</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>resolvable</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>tau_required_years</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="O1" s="27" t="inlineStr">
+        <is>
+          <t>consumer_quartz_unresolvable</t>
+        </is>
+      </c>
+      <c r="P1" s="27" t="inlineStr">
+        <is>
+          <t>link_limited_pairings</t>
+        </is>
+      </c>
+      <c r="Q1" s="27" t="inlineStr">
+        <is>
+          <t>claim_ceiling</t>
+        </is>
+      </c>
+      <c r="R1" s="27" t="inlineStr">
+        <is>
+          <t>bottleneck_note</t>
+        </is>
+      </c>
+      <c r="S1" s="27" t="inlineStr">
+        <is>
+          <t>why_run_it_anyway</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-QUARTZ_XO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>QUARTZ_XO</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>1.414213562373449e-09</v>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-QUARTZ_XO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>QUARTZ_XO</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>1.414213562373095e-09</v>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="7" t="n"/>
+      <c r="Q3" s="7" t="n"/>
+      <c r="R3" s="7" t="n"/>
+      <c r="S3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-TCXO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>TCXO</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>7.071067812572583e-11</v>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="7" t="n"/>
+      <c r="Q4" s="7" t="n"/>
+      <c r="R4" s="7" t="n"/>
+      <c r="S4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-TCXO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>TCXO</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>7.071067811865477e-11</v>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
+      <c r="Q5" s="7" t="n"/>
+      <c r="R5" s="7" t="n"/>
+      <c r="S5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OCXO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>OCXO</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>1.414248917270224e-13</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="7" t="n"/>
+      <c r="Q6" s="7" t="n"/>
+      <c r="R6" s="7" t="n"/>
+      <c r="S6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OCXO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>OCXO</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>1.414213562408451e-13</v>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
+      <c r="Q7" s="7" t="n"/>
+      <c r="R7" s="7" t="n"/>
+      <c r="S7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-RUBIDIUM-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>RUBIDIUM</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>1.417744687875783e-14</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-RUBIDIUM-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>RUBIDIUM</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>1.414213565908629e-14</v>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="n"/>
+      <c r="P9" s="7" t="n"/>
+      <c r="Q9" s="7" t="n"/>
+      <c r="R9" s="7" t="n"/>
+      <c r="S9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-GPSDO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>GPSDO</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>1.417744687875783e-14</v>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
+      <c r="Q10" s="7" t="n"/>
+      <c r="R10" s="7" t="n"/>
+      <c r="S10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-GPSDO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>GPSDO</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>1.414213565908629e-14</v>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
+      <c r="Q11" s="7" t="n"/>
+      <c r="R11" s="7" t="n"/>
+      <c r="S11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-CAESIUM-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>CAESIUM</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>1.732050807568877e-15</v>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>COMPARABLE_CONTRIBUTIONS</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
+      <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
+      <c r="S12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-CAESIUM-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>CAESIUM</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>1.414213915926442e-15</v>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
+      <c r="Q13" s="7" t="n"/>
+      <c r="R13" s="7" t="n"/>
+      <c r="S13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-HYDROGEN_MASER-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>HYDROGEN_MASER</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>1.009950493836208e-15</v>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>LINK_LIMITED</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="7" t="n"/>
+      <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="7" t="n"/>
+      <c r="S14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-HYDROGEN_MASER-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>HYDROGEN_MASER</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>1.414248917270224e-16</v>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>OSCILLATOR_LIMITED</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="7" t="n"/>
+      <c r="Q15" s="7" t="n"/>
+      <c r="R15" s="7" t="n"/>
+      <c r="S15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OPTICAL-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>OPTICAL</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>1.00000001e-15</v>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>LINK_LIMITED</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>UNRESOLVABLE_AT_ANY_INTEGRATION_TIME</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
+      <c r="Q16" s="7" t="n"/>
+      <c r="R16" s="7" t="n"/>
+      <c r="S16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OPTICAL-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>OPTICAL</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>1.091136967219822e-16</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>1.009950493836208e-18</v>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>LINK_LIMITED</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>5.323135106431327e-08</v>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>RESOLVABLE</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
+      <c r="Q17" s="7" t="n"/>
+      <c r="R17" s="7" t="n"/>
+      <c r="S17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-CEILING</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>claim_ceiling</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.ceiling_report</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="7" t="n"/>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>QUARTZ_XO; TCXO; OCXO</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>HYDROGEN_MASER+COAX_SHORT; OPTICAL+COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
+          <t>Two consumer quartz oscillators do not demonstrate metre-scale relativistic height sensing. Not because the experiment is hard, but because their flicker floor sits above the target and averaging does not lower a floor.</t>
+        </is>
+      </c>
+      <c r="R18" s="7" t="inlineStr">
+        <is>
+          <t>The limiting term moves. Consumer quartz is oscillator-limited and no link helps it. The best clocks are link-limited: an optical pair on short coax cannot resolve a metre, while the same pair on stabilized fibre resolves it in seconds. Buying a better clock without also buying a better link buys nothing.</t>
+        </is>
+      </c>
+      <c r="S18" s="7" t="inlineStr">
+        <is>
+          <t>The common-source split costs almost nothing and is the only way to learn what the measurement chain itself contributes. Every later claim depends on that number, and no amount of modelling substitutes for it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
+    <col width="54" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="27" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" s="27" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="D1" s="27" t="inlineStr">
+        <is>
+          <t>privacy_class</t>
+        </is>
+      </c>
+      <c r="E1" s="27" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="F1" s="27" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="G1" s="27" t="inlineStr">
+        <is>
+          <t>signed_by</t>
+        </is>
+      </c>
+      <c r="H1" s="27" t="inlineStr">
+        <is>
+          <t>signed_at</t>
+        </is>
+      </c>
+      <c r="I1" s="27" t="inlineStr">
+        <is>
+          <t>digest</t>
+        </is>
+      </c>
+      <c r="J1" s="27" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="K1" s="27" t="inlineStr">
+        <is>
+          <t>reversible</t>
+        </is>
+      </c>
+      <c r="L1" s="27" t="inlineStr">
+        <is>
+          <t>authorized_to_publish</t>
+        </is>
+      </c>
+      <c r="M1" s="27" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="N1" s="27" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="O1" s="27" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="P1" s="27" t="inlineStr">
+        <is>
+          <t>does_not_provide</t>
+        </is>
+      </c>
+      <c r="Q1" s="27" t="inlineStr">
+        <is>
+          <t>why_it_matters</t>
+        </is>
+      </c>
+      <c r="R1" s="27" t="inlineStr">
+        <is>
+          <t>preserves_patent_rights</t>
+        </is>
+      </c>
+      <c r="S1" s="27" t="inlineStr">
+        <is>
+          <t>creates_public_prior_art</t>
+        </is>
+      </c>
+      <c r="T1" s="27" t="inlineStr">
+        <is>
+          <t>forecloses</t>
+        </is>
+      </c>
+      <c r="U1" s="27" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>R7-PUBLICATION-DECISION</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>publication_decision</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.authorize_publication</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>PRIVATE_RC</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Andrew Green</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>f2f42c1ffde7d8922fb540fe8822f65a4268a0c9c2af216114049bc289667514</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7" t="inlineStr">
+        <is>
+          <t>PRIVATE_RC_NOTHING_PUBLISHED</t>
+        </is>
+      </c>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>PRIVATE_RC is a decision to publish nothing new. It is the only reversible option: FILE_THEN_PUBLISH and DEFENSIVE_PUBLICATION can both be chosen later, and neither can be undone once chosen.</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="n"/>
+      <c r="U2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>R7-COMMIT-IS-NOT-A-FILING</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>legal_boundary</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>r7.legacy.commit_is_not_a_filing</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="13" t="n"/>
+      <c r="H3" s="13" t="n"/>
+      <c r="I3" s="13" t="n"/>
+      <c r="J3" s="13" t="n"/>
+      <c r="K3" s="13" t="n"/>
+      <c r="L3" s="13" t="n"/>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>NOT_LEGAL_ADVICE</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="n"/>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>evidence of a date, if the repository history is preserved and trusted; a content hash that shows the text has not changed since</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>a patent filing or any priority date; a defensive publication in the legal sense; publication at all, while the repository is private; an enabling disclosure organized for a searcher to find; legal advice of any kind</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>A private repository discloses nothing, so it neither establishes prior art nor endangers novelty. Making it public is the act that does both at once -- it creates prior art against others and destroys novelty for the author. Those happen in the same instant and cannot be separated after the fact.</t>
+        </is>
+      </c>
+      <c r="R3" s="13" t="n"/>
+      <c r="S3" s="13" t="n"/>
+      <c r="T3" s="13" t="n"/>
+      <c r="U3" s="13" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>R7-PATH-FILE_THEN_PUBLISH</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>publication_path</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.path_comparison</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>FILE_THEN_PUBLISH</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n"/>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="7" t="n"/>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="7" t="n"/>
+      <c r="Q4" s="7" t="n"/>
+      <c r="R4" s="7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="S4" s="7" t="inlineStr">
+        <is>
+          <t>after filing</t>
+        </is>
+      </c>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>nothing, if filing precedes any disclosure</t>
+        </is>
+      </c>
+      <c r="U4" s="7" t="inlineStr">
+        <is>
+          <t>patent agent fees plus filing fees, per jurisdiction</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>R7-PATH-DEFENSIVE_PUBLICATION</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>publication_path</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.path_comparison</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>DEFENSIVE_PUBLICATION</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n"/>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="7" t="n"/>
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="7" t="n"/>
+      <c r="Q5" s="7" t="n"/>
+      <c r="R5" s="7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>immediately</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>the author's own ability to patent the disclosed subject matter in most jurisdictions</t>
+        </is>
+      </c>
+      <c r="U5" s="7" t="inlineStr">
+        <is>
+          <t>archival and preparation effort</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>R7-PATH-PRIVATE_RC</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>publication_path</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.path_comparison</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>PRIVATE_RC</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="7" t="n"/>
+      <c r="Q6" s="7" t="n"/>
+      <c r="R6" s="7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="U6" s="7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -17623,7 +20756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F237"/>
+  <dimension ref="A1:F272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24995,51 +28128,51 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="6" t="inlineStr">
-        <is>
-          <t>source_registry</t>
-        </is>
-      </c>
-      <c r="B231" s="6" t="inlineStr">
-        <is>
-          <t>SRC-V4X2-01</t>
-        </is>
-      </c>
-      <c r="C231" s="6" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D231" s="6" t="inlineStr">
-        <is>
-          <t>SOURCE_CLAIM</t>
-        </is>
-      </c>
-      <c r="E231" s="6" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F231" s="6" t="inlineStr">
-        <is>
-          <t>local hash 019435a03b3c5e9d</t>
+      <c r="A231" s="7" t="inlineStr">
+        <is>
+          <t>r7_cw</t>
+        </is>
+      </c>
+      <c r="B231" s="7" t="inlineStr">
+        <is>
+          <t>R7-CW-PARSE-NULL</t>
+        </is>
+      </c>
+      <c r="C231" s="7" t="inlineStr">
+        <is>
+          <t>parse_null</t>
+        </is>
+      </c>
+      <c r="D231" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E231" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F231" s="7" t="inlineStr">
+        <is>
+          <t>r7.cw.status_report</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r7_cw</t>
         </is>
       </c>
       <c r="B232" s="6" t="inlineStr">
         <is>
-          <t>SRC-V4X2-02</t>
+          <t>R7-CW-VECTOR-00</t>
         </is>
       </c>
       <c r="C232" s="6" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>source_vector</t>
         </is>
       </c>
       <c r="D232" s="6" t="inlineStr">
@@ -25054,24 +28187,24 @@
       </c>
       <c r="F232" s="6" t="inlineStr">
         <is>
-          <t>local hash 7e1df086615c6bac</t>
+          <t>JH corpus CW vector strings</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="6" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r7_cw</t>
         </is>
       </c>
       <c r="B233" s="6" t="inlineStr">
         <is>
-          <t>SRC-V4X2-03</t>
+          <t>R7-CW-VECTOR-01</t>
         </is>
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>source_vector</t>
         </is>
       </c>
       <c r="D233" s="6" t="inlineStr">
@@ -25086,24 +28219,24 @@
       </c>
       <c r="F233" s="6" t="inlineStr">
         <is>
-          <t>local hash b8e387558cb0a0f0</t>
+          <t>JH corpus CW vector strings</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="6" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r7_cw</t>
         </is>
       </c>
       <c r="B234" s="6" t="inlineStr">
         <is>
-          <t>SRC-V4X2-04</t>
+          <t>R7-CW-VECTOR-02</t>
         </is>
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>source_vector</t>
         </is>
       </c>
       <c r="D234" s="6" t="inlineStr">
@@ -25118,24 +28251,24 @@
       </c>
       <c r="F234" s="6" t="inlineStr">
         <is>
-          <t>local hash 473ab08fd766fe38</t>
+          <t>JH corpus CW vector strings</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="6" t="inlineStr">
         <is>
-          <t>source_registry</t>
+          <t>r7_cw</t>
         </is>
       </c>
       <c r="B235" s="6" t="inlineStr">
         <is>
-          <t>SRC-V4X2-05</t>
+          <t>R7-CW-VECTOR-03</t>
         </is>
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>source_vector</t>
         </is>
       </c>
       <c r="D235" s="6" t="inlineStr">
@@ -25150,69 +28283,1189 @@
       </c>
       <c r="F235" s="6" t="inlineStr">
         <is>
-          <t>local hash 32f952347682a67e</t>
+          <t>JH corpus CW vector strings</t>
         </is>
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="5" t="inlineStr">
-        <is>
-          <t>lore_registry</t>
-        </is>
-      </c>
-      <c r="B236" s="5" t="inlineStr">
-        <is>
-          <t>LORE-POLICY</t>
-        </is>
-      </c>
-      <c r="C236" s="5" t="inlineStr">
-        <is>
-          <t>lore_policy</t>
-        </is>
-      </c>
-      <c r="D236" s="5" t="inlineStr">
-        <is>
-          <t>LORE</t>
-        </is>
-      </c>
-      <c r="E236" s="5" t="inlineStr">
-        <is>
-          <t>PUBLIC_SAFE</t>
-        </is>
-      </c>
-      <c r="F236" s="5" t="inlineStr">
-        <is>
-          <t>docs/v4/resonator/LORE_AND_INTUITION_POLICY.md</t>
+      <c r="A236" s="6" t="inlineStr">
+        <is>
+          <t>r7_cw</t>
+        </is>
+      </c>
+      <c r="B236" s="6" t="inlineStr">
+        <is>
+          <t>R7-CW-VECTOR-04</t>
+        </is>
+      </c>
+      <c r="C236" s="6" t="inlineStr">
+        <is>
+          <t>source_vector</t>
+        </is>
+      </c>
+      <c r="D236" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E236" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F236" s="6" t="inlineStr">
+        <is>
+          <t>JH corpus CW vector strings</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="7" t="inlineStr">
         <is>
+          <t>r7_cw</t>
+        </is>
+      </c>
+      <c r="B237" s="7" t="inlineStr">
+        <is>
+          <t>R7-CW-DECODER-HEADER2_PLUS_3X12</t>
+        </is>
+      </c>
+      <c r="C237" s="7" t="inlineStr">
+        <is>
+          <t>frozen_decoder</t>
+        </is>
+      </c>
+      <c r="D237" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E237" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F237" s="7" t="inlineStr">
+        <is>
+          <t>r7.cw.FROZEN_DECODERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="7" t="inlineStr">
+        <is>
+          <t>r7_cw</t>
+        </is>
+      </c>
+      <c r="B238" s="7" t="inlineStr">
+        <is>
+          <t>R7-CW-DECODER-HEADER2_PLUS_6X6</t>
+        </is>
+      </c>
+      <c r="C238" s="7" t="inlineStr">
+        <is>
+          <t>frozen_decoder</t>
+        </is>
+      </c>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E238" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F238" s="7" t="inlineStr">
+        <is>
+          <t>r7.cw.FROZEN_DECODERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="7" t="inlineStr">
+        <is>
+          <t>r7_gravity</t>
+        </is>
+      </c>
+      <c r="B239" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-HANDHELD_CRYSTAL</t>
+        </is>
+      </c>
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="D239" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E239" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F239" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="7" t="inlineStr">
+        <is>
+          <t>r7_gravity</t>
+        </is>
+      </c>
+      <c r="B240" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-BENCH_COIL_DRIVE</t>
+        </is>
+      </c>
+      <c r="C240" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="D240" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E240" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F240" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="7" t="inlineStr">
+        <is>
+          <t>r7_gravity</t>
+        </is>
+      </c>
+      <c r="B241" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-HIGH_POWER_PULSE</t>
+        </is>
+      </c>
+      <c r="C241" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="D241" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E241" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F241" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="7" t="inlineStr">
+        <is>
+          <t>r7_gravity</t>
+        </is>
+      </c>
+      <c r="B242" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-ABSURD_UPPER_BOUND</t>
+        </is>
+      </c>
+      <c r="C242" s="7" t="inlineStr">
+        <is>
+          <t>gravity_arithmetic</t>
+        </is>
+      </c>
+      <c r="D242" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E242" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F242" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.assess</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="7" t="inlineStr">
+        <is>
+          <t>r7_gravity</t>
+        </is>
+      </c>
+      <c r="B243" s="7" t="inlineStr">
+        <is>
+          <t>R7-GRAVITY-VERDICT</t>
+        </is>
+      </c>
+      <c r="C243" s="7" t="inlineStr">
+        <is>
+          <t>gravity_verdict</t>
+        </is>
+      </c>
+      <c r="D243" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E243" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F243" s="7" t="inlineStr">
+        <is>
+          <t>r7.gravity.full_assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B244" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-QUARTZ_XO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C244" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D244" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E244" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F244" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B245" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-QUARTZ_XO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C245" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D245" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E245" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F245" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B246" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-TCXO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C246" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D246" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E246" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F246" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B247" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-TCXO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C247" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D247" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E247" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F247" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B248" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OCXO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C248" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D248" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E248" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F248" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B249" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OCXO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C249" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D249" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E249" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F249" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B250" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-RUBIDIUM-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C250" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D250" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E250" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F250" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B251" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-RUBIDIUM-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C251" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D251" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E251" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F251" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B252" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-GPSDO-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C252" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D252" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E252" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F252" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B253" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-GPSDO-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C253" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D253" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E253" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F253" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B254" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-CAESIUM-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C254" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D254" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E254" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F254" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B255" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-CAESIUM-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C255" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D255" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E255" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F255" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B256" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-HYDROGEN_MASER-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C256" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D256" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E256" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F256" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B257" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-HYDROGEN_MASER-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C257" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D257" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E257" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F257" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B258" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OPTICAL-COAX_SHORT</t>
+        </is>
+      </c>
+      <c r="C258" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D258" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E258" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F258" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B259" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-OPTICAL-FIBRE_STABILIZED</t>
+        </is>
+      </c>
+      <c r="C259" s="7" t="inlineStr">
+        <is>
+          <t>height_resolution</t>
+        </is>
+      </c>
+      <c r="D259" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E259" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F259" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.height_resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="7" t="inlineStr">
+        <is>
+          <t>r7_clocklink</t>
+        </is>
+      </c>
+      <c r="B260" s="7" t="inlineStr">
+        <is>
+          <t>R7-CLOCK-CEILING</t>
+        </is>
+      </c>
+      <c r="C260" s="7" t="inlineStr">
+        <is>
+          <t>claim_ceiling</t>
+        </is>
+      </c>
+      <c r="D260" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E260" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F260" s="7" t="inlineStr">
+        <is>
+          <t>r7.clocklink.ceiling_report</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="7" t="inlineStr">
+        <is>
+          <t>r7_governance</t>
+        </is>
+      </c>
+      <c r="B261" s="7" t="inlineStr">
+        <is>
+          <t>R7-PUBLICATION-DECISION</t>
+        </is>
+      </c>
+      <c r="C261" s="7" t="inlineStr">
+        <is>
+          <t>publication_decision</t>
+        </is>
+      </c>
+      <c r="D261" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E261" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F261" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.authorize_publication</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="13" t="inlineStr">
+        <is>
+          <t>r7_governance</t>
+        </is>
+      </c>
+      <c r="B262" s="13" t="inlineStr">
+        <is>
+          <t>R7-COMMIT-IS-NOT-A-FILING</t>
+        </is>
+      </c>
+      <c r="C262" s="13" t="inlineStr">
+        <is>
+          <t>legal_boundary</t>
+        </is>
+      </c>
+      <c r="D262" s="13" t="inlineStr">
+        <is>
+          <t>UNSUPPORTED</t>
+        </is>
+      </c>
+      <c r="E262" s="13" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F262" s="13" t="inlineStr">
+        <is>
+          <t>r7.legacy.commit_is_not_a_filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="7" t="inlineStr">
+        <is>
+          <t>r7_governance</t>
+        </is>
+      </c>
+      <c r="B263" s="7" t="inlineStr">
+        <is>
+          <t>R7-PATH-FILE_THEN_PUBLISH</t>
+        </is>
+      </c>
+      <c r="C263" s="7" t="inlineStr">
+        <is>
+          <t>publication_path</t>
+        </is>
+      </c>
+      <c r="D263" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E263" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F263" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.path_comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="7" t="inlineStr">
+        <is>
+          <t>r7_governance</t>
+        </is>
+      </c>
+      <c r="B264" s="7" t="inlineStr">
+        <is>
+          <t>R7-PATH-DEFENSIVE_PUBLICATION</t>
+        </is>
+      </c>
+      <c r="C264" s="7" t="inlineStr">
+        <is>
+          <t>publication_path</t>
+        </is>
+      </c>
+      <c r="D264" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E264" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F264" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.path_comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="7" t="inlineStr">
+        <is>
+          <t>r7_governance</t>
+        </is>
+      </c>
+      <c r="B265" s="7" t="inlineStr">
+        <is>
+          <t>R7-PATH-PRIVATE_RC</t>
+        </is>
+      </c>
+      <c r="C265" s="7" t="inlineStr">
+        <is>
+          <t>publication_path</t>
+        </is>
+      </c>
+      <c r="D265" s="7" t="inlineStr">
+        <is>
+          <t>DERIVED_ARITHMETIC</t>
+        </is>
+      </c>
+      <c r="E265" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F265" s="7" t="inlineStr">
+        <is>
+          <t>r7.legacy.path_comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B266" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-01</t>
+        </is>
+      </c>
+      <c r="C266" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D266" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E266" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F266" s="6" t="inlineStr">
+        <is>
+          <t>local hash 019435a03b3c5e9d</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B267" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-02</t>
+        </is>
+      </c>
+      <c r="C267" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D267" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E267" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F267" s="6" t="inlineStr">
+        <is>
+          <t>local hash 7e1df086615c6bac</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B268" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-03</t>
+        </is>
+      </c>
+      <c r="C268" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D268" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E268" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F268" s="6" t="inlineStr">
+        <is>
+          <t>local hash b8e387558cb0a0f0</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B269" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-04</t>
+        </is>
+      </c>
+      <c r="C269" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D269" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E269" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F269" s="6" t="inlineStr">
+        <is>
+          <t>local hash 473ab08fd766fe38</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="6" t="inlineStr">
+        <is>
+          <t>source_registry</t>
+        </is>
+      </c>
+      <c r="B270" s="6" t="inlineStr">
+        <is>
+          <t>SRC-V4X2-05</t>
+        </is>
+      </c>
+      <c r="C270" s="6" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="D270" s="6" t="inlineStr">
+        <is>
+          <t>SOURCE_CLAIM</t>
+        </is>
+      </c>
+      <c r="E270" s="6" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F270" s="6" t="inlineStr">
+        <is>
+          <t>local hash 32f952347682a67e</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="5" t="inlineStr">
+        <is>
+          <t>lore_registry</t>
+        </is>
+      </c>
+      <c r="B271" s="5" t="inlineStr">
+        <is>
+          <t>LORE-POLICY</t>
+        </is>
+      </c>
+      <c r="C271" s="5" t="inlineStr">
+        <is>
+          <t>lore_policy</t>
+        </is>
+      </c>
+      <c r="D271" s="5" t="inlineStr">
+        <is>
+          <t>LORE</t>
+        </is>
+      </c>
+      <c r="E271" s="5" t="inlineStr">
+        <is>
+          <t>PUBLIC_SAFE</t>
+        </is>
+      </c>
+      <c r="F271" s="5" t="inlineStr">
+        <is>
+          <t>docs/v4/resonator/LORE_AND_INTUITION_POLICY.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="7" t="inlineStr">
+        <is>
           <t>installer_metadata</t>
         </is>
       </c>
-      <c r="B237" s="7" t="inlineStr">
+      <c r="B272" s="7" t="inlineStr">
         <is>
           <t>REL-v4.5.0</t>
         </is>
       </c>
-      <c r="C237" s="7" t="inlineStr">
+      <c r="C272" s="7" t="inlineStr">
         <is>
           <t>release_metadata</t>
         </is>
       </c>
-      <c r="D237" s="7" t="inlineStr">
+      <c r="D272" s="7" t="inlineStr">
         <is>
           <t>DERIVED_ARITHMETIC</t>
         </is>
       </c>
-      <c r="E237" s="7" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
-      <c r="F237" s="7" t="inlineStr">
+      <c r="E272" s="7" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="F272" s="7" t="inlineStr">
         <is>
           <t>pyproject.toml + build</t>
         </is>

</xml_diff>

<commit_message>
v5.2.1: version bump, release notes, and workbook
Supersedes v5.2.0, whose CI was red because the packaging guard could
not collect without setuptools (R9-D-020). The v5.2.0 tag is immutable
and stays as cut; the release notes for v5.2.1 say plainly why it
exists rather than quietly replacing it.

Release notes track the current version in the count guard, per the
convention added at v5.2.0: superseded notes are frozen at the count
that was true when they shipped.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.2.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.2.1 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.2.0</t>
+          <t>5.2.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.3.0: release metadata, evidence workbook, and version bump
Clean-clone count 2564 -> 2708. Version 5.2.1 -> 5.3.0 across
pyproject, CITATION.cff, README and the guard constants; workbook
regenerated and its SHA256SUMS entry updated; release gate returns
TAG_MAY_PROCEED.

Minor bump rather than patch: r10 adds new public modules
(cwarith, cwontology, energyledger, unruh, firewall) without breaking
anything existing.

The count guard is repointed at the v5.3.0 notes, per the convention
established at v5.2.0 -- superseded release notes stay frozen at the
count that was true when they shipped rather than being rewritten to
satisfy the guard.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.2.1 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.3.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.2.1</t>
+          <t>5.3.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.3.1: release metadata, workbook, and the count set to 2808
2807 was measured with the count guard still failing on a placeholder;
fixing it makes that test pass, so the figure is 2808. Applied from
the recorded lesson rather than rediscovered.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.3.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.3.1 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.3.0</t>
+          <t>5.3.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.4.0: release metadata, workbook, count 2837
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.3.1 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.4.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.3.1</t>
+          <t>5.4.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.4.1: release metadata, workbook, count 2867
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.4.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.4.1 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.4.0</t>
+          <t>5.4.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.5.0: release metadata, workbook, count 2948
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.4.1 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.5.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.4.1</t>
+          <t>5.5.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.6.0: release metadata, workbook, count 3014
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.5.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.6.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.5.0</t>
+          <t>5.6.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.7.0: version bump, release notes, changelog, metadata, workbook, count 3079
- pyproject/CITATION/README bumped to 5.7.0 (date-released 2026-07-23)
- RELEASE_NOTES_V5_7_0.md + CHANGELOG [5.7.0] entry
- release metadata authority refreshed to 3079 passed / 1 deselected
  (full suite, policy D-V3-04 deselect); all documented count sites agree
- workbook + SHA256SUMS regenerated; release gate TAG_MAY_PROCEED
- guard tests and metadata COUNT_SITES repointed to v5.7.0

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.6.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.7.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.6.0</t>
+          <t>5.7.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.8.0: version bump, release notes, changelog, metadata, workbook, count 3340
- pyproject/CITATION/README bumped to 5.8.0
- RELEASE_NOTES_V5_8_0.md + CHANGELOG [5.8.0] entry
- release metadata refreshed to 3340 passed / 1 deselected (full local
  suite on the exact commit; all documented count sites agree)
- workbook + SHA256SUMS regenerated; release gate TAG_MAY_PROCEED
- guard tests and metadata COUNT_SITES repointed to v5.8.0
- CI unavailable (free-tier Actions minutes exhausted); local suite is
  the verification of record

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.7.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.8.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.7.0</t>
+          <t>5.8.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.9.0: version bump, release notes, changelog, metadata, workbook, count 3485
- pyproject/CITATION/README bumped to 5.9.0
- RELEASE_NOTES_V5_9_0.md + CHANGELOG [5.9.0] entry
- release metadata refreshed to 3485 passed / 1 deselected (full local
  suite on the exact commit, all gates green; documented count sites agree)
- workbook + SHA256SUMS regenerated; release gate TAG_MAY_PROCEED
- guard tests and metadata COUNT_SITES repointed to v5.9.0
- CI unavailable (free-tier Actions minutes exhausted); local suite is the
  verification of record

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.8.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v5.9.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.8.0</t>
+          <t>5.9.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v6.0.0: version bump, release notes, changelog, metadata, workbook, count 4062
- pyproject/CITATION/README bumped to 6.0.0 (major: r11 is a new public
  package and tests/v6 a new suite root)
- docs/v6/RELEASE_NOTES_V6_0_0.md + CHANGELOG [6.0.0] entry
- release metadata measured on the FULLY GREEN suite: 4062 passed,
  1 deselected, 0 failed, exit 0; all documented count sites agree
- workbook + SHA256SUMS regenerated; release gate TAG_MAY_PROCEED
- guard tests and metadata COUNT_SITES repointed to v6.0.0
- CI unavailable (free-tier Actions minutes exhausted); local suite on the
  exact commit is the verification of record

Verdict: R11_GREEN_MODELS_IMPLEMENTED_DECODER_NOT_IDENTIFIED.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v5.9.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v6.0.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>5.9.0</t>
+          <t>6.0.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v6.1.0: version bump, delta findings, release notes, changelog, count 4412
- pyproject/CITATION/README bumped to 6.1.0
- docs/v6/R11_DELTA_FINDINGS.md + RELEASE_NOTES_V6_1_0.md + CHANGELOG entry
- release metadata measured on the FULLY GREEN suite: 4412 passed,
  1 deselected, 0 failed, exit 0; all documented count sites agree
- workbook + SHA256SUMS regenerated; release gate TAG_MAY_PROCEED
- CI unavailable (free-tier Actions minutes exhausted); local suite on the
  exact commit is the verification of record

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v6.0.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v6.1.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>6.0.0</t>
+          <t>6.1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v6.2.0: R11.1 findings, release notes, changelog, count 4936
- pyproject/CITATION/README bumped to 6.2.0 (the pack proposed v6.1.0, but
  that had already shipped)
- docs/v6/R11_1_FINDINGS.md + RELEASE_NOTES_V6_2_0.md + CHANGELOG entry
- release metadata 4936 passed / 1 deselected; all documented count sites
  agree; workbook + SHA256SUMS regenerated; gate TAG_MAY_PROCEED
- private_do_not_commit/ never read and never tracked

Verdict: R11_1_GREEN_MODELS_AND_EXPERIMENTS_IMPLEMENTED_NO_NEW_PHYSICS_CLAIM

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v6.1.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v6.2.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>6.1.0</t>
+          <t>6.2.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v6.3.0: R12 findings, release notes, changelog, count 5175
- pyproject/CITATION/README bumped to 6.3.0
- docs/v6/R12_FINDINGS.md + RELEASE_NOTES_V6_3_0.md + CHANGELOG entry
- release metadata 5175 passed / 1 deselected; all documented count sites
  agree; workbook + SHA256SUMS regenerated; gate TAG_MAY_PROCEED
- private_do_not_commit/ never read and never tracked

Verdict: R12_GREEN_ICOSAHEDRAL_AND_BRIDGE_ARCHITECTURE_IMPLEMENTED_NO_UNIQUE_DECODE

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/release/v45/RGCS_Master_Evidence_Workbook.xlsx
+++ b/release/v45/RGCS_Master_Evidence_Workbook.xlsx
@@ -1505,7 +1505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schema 1.0.0 · RGCS v6.2.0 · generated from canonical repository data</t>
+          <t>Schema 1.0.0 · RGCS v6.3.0 · generated from canonical repository data</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>6.2.0</t>
+          <t>6.3.0</t>
         </is>
       </c>
     </row>

</xml_diff>